<commit_message>
ACT NO.3 ( Pkhanh)
</commit_message>
<xml_diff>
--- a/Template_PRJ301_AI_Usage_Report_Template 10.xlsx
+++ b/Template_PRJ301_AI_Usage_Report_Template 10.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LAPTOP\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\COLLEGE\FALL26\PRJ201\aita-plagiarism-detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{076E364D-431E-4896-9CA8-0C0159D13083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E232C902-5BE0-44F5-B6B3-79767205A716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0.Overview" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="89">
   <si>
     <t>PRJ301 - Project AI Usage Report</t>
   </si>
@@ -269,6 +269,30 @@
   </si>
   <si>
     <t>AI failed to deeply understand the project's specific "academic market" logic and point-payment mechanism, resulting in a generic schema that required manual adjustments.</t>
+  </si>
+  <si>
+    <t>Requirement</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find the actors may have in the system and see what usecases is appropriate in the system, Also generated SRS (Specification requi  file </t>
+  </si>
+  <si>
+    <t>Proposed a structure of 5 actor participate in the system (Student, lecture, systemadministrator, AI Similarity Engine and Acaedmic council) with some of use case  for each actor, it also give a SRS document about 11 pages.</t>
+  </si>
+  <si>
+    <t>Removed 2 secondary actors (AI Similarity Engine and Conference Council) and replace it with 2 new actor are External AI Service and AITA Submisson Portal acording to context of the system. (This is just my subjective opinion - chủ quan).</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1zzjKhSxxiEcWQbvnrOPi1hP_8b1GvXZD?usp=sharing</t>
+  </si>
+  <si>
+    <t>3 actors integrated in system finalized ver 1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Although give specific context but AI still not fully understand the system and have some wrong external resulting identify wrong actors in the system. Also the SRS document pernamently still not haven't detected error but still need to follow up. </t>
   </si>
 </sst>
 </file>
@@ -356,7 +380,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -403,12 +427,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -437,19 +489,37 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -756,108 +826,108 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="14">
         <v>7</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="15"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="13"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>12</v>
       </c>
@@ -874,7 +944,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="4">
         <v>1</v>
       </c>
@@ -887,7 +957,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="4">
         <v>2</v>
       </c>
@@ -900,7 +970,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="4">
         <v>3</v>
       </c>
@@ -913,7 +983,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="4">
         <v>4</v>
       </c>
@@ -926,7 +996,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="4">
         <v>5</v>
       </c>
@@ -957,22 +1027,22 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="23.796875" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="24.88671875" customWidth="1"/>
+    <col min="7" max="7" width="24.86328125" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="61.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>17</v>
       </c>
@@ -1004,7 +1074,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="68.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1023,7 +1093,7 @@
       <c r="F2" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="10" t="s">
         <v>73</v>
       </c>
       <c r="H2" s="6" t="s">
@@ -1036,36 +1106,68 @@
         <v>75</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+    <row r="3" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="17">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="17">
         <v>4</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="18" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="123" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="20">
+        <v>3</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="20">
+        <v>1</v>
+      </c>
+      <c r="J4" s="21" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1080,7 +1182,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1094,7 +1196,7 @@
     <col min="10" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>17</v>
       </c>
@@ -1126,7 +1228,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1158,7 +1260,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1198,13 +1300,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
         <v>44</v>
       </c>
@@ -1212,7 +1314,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>17</v>
       </c>
@@ -1220,7 +1322,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>18</v>
       </c>
@@ -1228,7 +1330,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>19</v>
       </c>
@@ -1236,7 +1338,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" s="8" t="s">
         <v>20</v>
       </c>
@@ -1244,7 +1346,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>21</v>
       </c>
@@ -1252,7 +1354,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
         <v>22</v>
       </c>
@@ -1260,7 +1362,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="38.25" x14ac:dyDescent="0.45">
       <c r="A8" s="8" t="s">
         <v>23</v>
       </c>
@@ -1268,7 +1370,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A9" s="8" t="s">
         <v>24</v>
       </c>
@@ -1276,7 +1378,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" s="8" t="s">
         <v>25</v>
       </c>
@@ -1284,7 +1386,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
         <v>26</v>
       </c>

</xml_diff>

<commit_message>
Xóa file 36 log AI
</commit_message>
<xml_diff>
--- a/Template_PRJ301_AI_Usage_Report_Template 10.xlsx
+++ b/Template_PRJ301_AI_Usage_Report_Template 10.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phucv\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\COLLEGE\FALL26\PRJ201\aita-plagiarism-detection\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB9FDE2B-BFC6-4385-BB99-BD34D6713374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9204" activeTab="1"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0.Overview" sheetId="1" r:id="rId1"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="126">
   <si>
     <t>PRJ301 - Project AI Usage Report</t>
   </si>
@@ -379,12 +380,36 @@
   </si>
   <si>
     <t>AI omitted asynchronous processing limits, so manual intervention was needed to specify how long-running plagiarism checks interact with Servlet HTTP timeout limits.</t>
+  </si>
+  <si>
+    <t>Requirement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find the actors may have in the system and see what usecases is appropriate in the system, Also generated SRS (Specification requi  file </t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>Proposed a structure of 5 actor participate in the system (Student, lecture, systemadministrator, AI Similarity Engine and Acaedmic council) with some of use case  for each actor, it also give a SRS document about 11 pages.</t>
+  </si>
+  <si>
+    <t>Removed 2 secondary actors (AI Similarity Engine and Conference Council) and replace it with 2 new actor are External AI Service and AITA Submisson Portal acording to context of the system. (This is just my subjective opinion - chủ quan).</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/drive/folders/1zzjKhSxxiEcWQbvnrOPi1hP_8b1GvXZD?usp=sharing</t>
+  </si>
+  <si>
+    <t>3 actors integrated in system finalized ver 1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Although give specific context but AI still not fully understand the system and have some wrong external resulting identify wrong actors in the system. Also the SRS document pernamently still not haven't detected error but still need to follow up. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -472,7 +497,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -519,12 +544,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -559,30 +612,31 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -885,110 +939,110 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="14"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="15"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="14"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="14"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="14"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="15"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="14"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="15"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="16">
         <v>7</v>
       </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="14"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="14"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="16" t="s">
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="15"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="14"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="15"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>15</v>
       </c>
@@ -1005,7 +1059,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A13" s="4">
         <v>1</v>
       </c>
@@ -1018,7 +1072,7 @@
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A14" s="4">
         <v>2</v>
       </c>
@@ -1031,7 +1085,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A15" s="4">
         <v>3</v>
       </c>
@@ -1044,7 +1098,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A16" s="4">
         <v>4</v>
       </c>
@@ -1059,7 +1113,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="4">
         <v>5</v>
       </c>
@@ -1089,9 +1143,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:J10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="23.6640625" customWidth="1"/>
@@ -1099,13 +1153,13 @@
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="26" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="24.88671875" customWidth="1"/>
+    <col min="7" max="7" width="24.86328125" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="61.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
@@ -1137,7 +1191,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="68.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1169,7 +1223,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1201,7 +1255,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1233,7 +1287,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1265,7 +1319,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="84" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1297,7 +1351,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="92.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="89.25" x14ac:dyDescent="0.45">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1329,85 +1383,117 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="105.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="18">
+    <row r="8" spans="1:10" ht="102" x14ac:dyDescent="0.45">
+      <c r="A8" s="5">
         <v>7</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="G8" s="17" t="s">
+      <c r="G8" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="I8" s="18">
+      <c r="I8" s="5">
         <v>5</v>
       </c>
-      <c r="J8" s="19" t="s">
+      <c r="J8" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="92.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="20">
+    <row r="9" spans="1:10" ht="89.25" x14ac:dyDescent="0.45">
+      <c r="A9" s="18">
         <v>8</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="19" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="19" t="s">
         <v>114</v>
       </c>
-      <c r="F9" s="21" t="s">
+      <c r="F9" s="19" t="s">
         <v>115</v>
       </c>
-      <c r="G9" s="17" t="s">
+      <c r="G9" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="19" t="s">
         <v>116</v>
       </c>
-      <c r="I9" s="20">
+      <c r="I9" s="18">
         <v>4</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="19" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="114.75" x14ac:dyDescent="0.45">
+      <c r="A10" s="20">
+        <v>9</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>119</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="H10" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="I10" s="20">
+        <v>1</v>
+      </c>
+      <c r="J10" s="21" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1"/>
-    <hyperlink ref="G3" r:id="rId2"/>
-    <hyperlink ref="G8" r:id="rId3"/>
-    <hyperlink ref="G9" r:id="rId4"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="G8" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="G9" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -1421,7 +1507,7 @@
     <col min="10" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
@@ -1453,7 +1539,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="39.6" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1485,7 +1571,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1523,15 +1609,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="7" t="s">
         <v>76</v>
       </c>
@@ -1539,7 +1625,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="8" t="s">
         <v>29</v>
       </c>
@@ -1547,7 +1633,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>30</v>
       </c>
@@ -1555,7 +1641,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>31</v>
       </c>
@@ -1563,7 +1649,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" s="8" t="s">
         <v>32</v>
       </c>
@@ -1571,7 +1657,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="8" t="s">
         <v>33</v>
       </c>
@@ -1579,7 +1665,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
         <v>34</v>
       </c>
@@ -1587,7 +1673,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="39.6" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="8" t="s">
         <v>35</v>
       </c>
@@ -1595,7 +1681,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="8" t="s">
         <v>36</v>
       </c>
@@ -1603,7 +1689,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" s="8" t="s">
         <v>37</v>
       </c>
@@ -1611,7 +1697,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="26.45" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="8" t="s">
         <v>38</v>
       </c>

</xml_diff>